<commit_message>
Korjaa t0_50p_liukuva laskemaan mean([t-49...t0]) / t0_low × 100 dokumentaation mukaisesti.
</commit_message>
<xml_diff>
--- a/data/results.xlsx
+++ b/data/results.xlsx
@@ -985,19 +985,19 @@
         <v>103.46</v>
       </c>
       <c r="V2" s="2" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="W2" s="2" t="n">
-        <v>2.35</v>
+        <v>2.1</v>
       </c>
       <c r="X2" s="2" t="n">
-        <v>1.87</v>
+        <v>1.78</v>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>1.61</v>
+        <v>1.56</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>1.84</v>
+        <v>1.79</v>
       </c>
       <c r="AA2" s="2" t="n">
         <v>102.85</v>
@@ -1227,19 +1227,19 @@
         <v>97.91</v>
       </c>
       <c r="V3" s="2" t="n">
-        <v>1.84</v>
+        <v>1.3</v>
       </c>
       <c r="W3" s="2" t="n">
-        <v>1.01</v>
+        <v>0.9</v>
       </c>
       <c r="X3" s="2" t="n">
-        <v>1.7</v>
+        <v>1.61</v>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>1.64</v>
+        <v>1.58</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>2.37</v>
+        <v>2.31</v>
       </c>
       <c r="AA3" s="2" t="n">
         <v>101.22</v>
@@ -1471,19 +1471,19 @@
         <v>94.44</v>
       </c>
       <c r="V4" s="2" t="n">
-        <v>1.44</v>
+        <v>1.02</v>
       </c>
       <c r="W4" s="2" t="n">
-        <v>0.93</v>
+        <v>0.83</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>1.58</v>
+        <v>1.5</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>1.92</v>
+        <v>1.88</v>
       </c>
       <c r="AA4" s="2" t="n">
         <v>101.99</v>
@@ -1715,19 +1715,19 @@
         <v>104.35</v>
       </c>
       <c r="V5" s="2" t="n">
-        <v>0.2</v>
+        <v>0.14</v>
       </c>
       <c r="W5" s="2" t="n">
-        <v>0.62</v>
+        <v>0.55</v>
       </c>
       <c r="X5" s="2" t="n">
-        <v>1.49</v>
+        <v>1.41</v>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>1.55</v>
+        <v>1.5</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>1.76</v>
+        <v>1.71</v>
       </c>
       <c r="AA5" s="2" t="n">
         <v>103.57</v>
@@ -1959,19 +1959,19 @@
         <v>106.9</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>1.12</v>
+        <v>0.79</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.33</v>
+        <v>1.19</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>2.87</v>
+        <v>2.73</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>3.32</v>
+        <v>3.21</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>3.01</v>
+        <v>2.93</v>
       </c>
       <c r="AA6" s="2" t="n">
         <v>103.14</v>
@@ -2203,19 +2203,19 @@
         <v>96.14</v>
       </c>
       <c r="V7" s="2" t="n">
-        <v>0.4</v>
+        <v>0.29</v>
       </c>
       <c r="W7" s="2" t="n">
-        <v>0.57</v>
+        <v>0.51</v>
       </c>
       <c r="X7" s="2" t="n">
-        <v>1.46</v>
+        <v>1.39</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <v>1.34</v>
+        <v>1.29</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>1.44</v>
+        <v>1.4</v>
       </c>
       <c r="AA7" s="2" t="n">
         <v>103.88</v>
@@ -2449,19 +2449,19 @@
         <v>94.79000000000001</v>
       </c>
       <c r="V8" s="2" t="n">
-        <v>0.31</v>
+        <v>0.22</v>
       </c>
       <c r="W8" s="2" t="n">
-        <v>1.72</v>
+        <v>1.53</v>
       </c>
       <c r="X8" s="2" t="n">
-        <v>1.86</v>
+        <v>1.76</v>
       </c>
       <c r="Y8" s="2" t="n">
-        <v>2.36</v>
+        <v>2.28</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>2.28</v>
+        <v>2.22</v>
       </c>
       <c r="AA8" s="2" t="n">
         <v>100.39</v>
@@ -2695,19 +2695,19 @@
         <v>81.22</v>
       </c>
       <c r="V9" s="2" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="W9" s="2" t="n">
-        <v>0.41</v>
+        <v>0.37</v>
       </c>
       <c r="X9" s="2" t="n">
-        <v>2.27</v>
+        <v>2.15</v>
       </c>
       <c r="Y9" s="2" t="n">
-        <v>7.41</v>
+        <v>7.16</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>8.380000000000001</v>
+        <v>8.16</v>
       </c>
       <c r="AA9" s="2" t="n">
         <v>100.35</v>
@@ -2941,19 +2941,19 @@
         <v>98.14</v>
       </c>
       <c r="V10" s="2" t="n">
-        <v>0.54</v>
+        <v>0.38</v>
       </c>
       <c r="W10" s="2" t="n">
-        <v>1.19</v>
+        <v>1.07</v>
       </c>
       <c r="X10" s="2" t="n">
-        <v>1.51</v>
+        <v>1.43</v>
       </c>
       <c r="Y10" s="2" t="n">
-        <v>1.26</v>
+        <v>1.21</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>1.2</v>
+        <v>1.17</v>
       </c>
       <c r="AA10" s="2" t="n">
         <v>100.92</v>
@@ -3187,19 +3187,19 @@
         <v>99.34</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>1.04</v>
+        <v>0.73</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>0.84</v>
+        <v>0.75</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>0.85</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>1.25</v>
+        <v>1.22</v>
       </c>
       <c r="AA11" s="2" t="n">
         <v>98.13</v>
@@ -3433,19 +3433,19 @@
         <v>100.77</v>
       </c>
       <c r="V12" s="2" t="n">
-        <v>1.12</v>
+        <v>0.79</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>1.69</v>
+        <v>1.64</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>2.12</v>
+        <v>2.06</v>
       </c>
       <c r="AA12" s="2" t="n">
         <v>100.11</v>
@@ -3679,19 +3679,19 @@
         <v>87.75</v>
       </c>
       <c r="V13" s="2" t="n">
-        <v>1.31</v>
+        <v>0.93</v>
       </c>
       <c r="W13" s="2" t="n">
-        <v>1.42</v>
+        <v>1.27</v>
       </c>
       <c r="X13" s="2" t="n">
-        <v>5.49</v>
+        <v>5.21</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>7.41</v>
+        <v>7.15</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>7.25</v>
+        <v>7.07</v>
       </c>
       <c r="AA13" s="2" t="n">
         <v>101.55</v>
@@ -3925,19 +3925,19 @@
         <v>89.77</v>
       </c>
       <c r="V14" s="2" t="n">
-        <v>1.18</v>
+        <v>0.83</v>
       </c>
       <c r="W14" s="2" t="n">
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
       <c r="X14" s="2" t="n">
-        <v>1.37</v>
+        <v>1.3</v>
       </c>
       <c r="Y14" s="2" t="n">
-        <v>2.15</v>
+        <v>2.07</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>3.49</v>
+        <v>3.4</v>
       </c>
       <c r="AA14" s="2" t="n">
         <v>102.05</v>
@@ -4171,19 +4171,19 @@
         <v>91.98</v>
       </c>
       <c r="V15" s="2" t="n">
-        <v>0.84</v>
+        <v>0.59</v>
       </c>
       <c r="W15" s="2" t="n">
-        <v>1.34</v>
+        <v>1.2</v>
       </c>
       <c r="X15" s="2" t="n">
-        <v>2.07</v>
+        <v>1.97</v>
       </c>
       <c r="Y15" s="2" t="n">
-        <v>2.53</v>
+        <v>2.44</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>3.33</v>
+        <v>3.25</v>
       </c>
       <c r="AA15" s="2" t="n">
         <v>104.27</v>
@@ -4417,19 +4417,19 @@
         <v>93.77</v>
       </c>
       <c r="V16" s="2" t="n">
-        <v>0.51</v>
+        <v>0.36</v>
       </c>
       <c r="W16" s="2" t="n">
-        <v>0.61</v>
+        <v>0.54</v>
       </c>
       <c r="X16" s="2" t="n">
-        <v>1.17</v>
+        <v>1.11</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>1.73</v>
+        <v>1.68</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>2.46</v>
+        <v>2.4</v>
       </c>
       <c r="AA16" s="2" t="n">
         <v>108.53</v>
@@ -4663,19 +4663,19 @@
         <v>84.14</v>
       </c>
       <c r="V17" s="2" t="n">
-        <v>1.01</v>
+        <v>0.72</v>
       </c>
       <c r="W17" s="2" t="n">
-        <v>1.17</v>
+        <v>1.05</v>
       </c>
       <c r="X17" s="2" t="n">
-        <v>1.61</v>
+        <v>1.52</v>
       </c>
       <c r="Y17" s="2" t="n">
-        <v>5.64</v>
+        <v>5.45</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>7.75</v>
+        <v>7.55</v>
       </c>
       <c r="AA17" s="2" t="n">
         <v>104.16</v>
@@ -4909,19 +4909,19 @@
         <v>105.69</v>
       </c>
       <c r="V18" s="2" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="W18" s="2" t="n">
-        <v>3.94</v>
+        <v>3.53</v>
       </c>
       <c r="X18" s="2" t="n">
-        <v>3.46</v>
+        <v>3.28</v>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>3.61</v>
+        <v>3.49</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>5.51</v>
+        <v>5.37</v>
       </c>
       <c r="AA18" s="2" t="n">
         <v>101.59</v>
@@ -5155,19 +5155,19 @@
         <v>108.02</v>
       </c>
       <c r="V19" s="2" t="n">
-        <v>0.28</v>
+        <v>0.2</v>
       </c>
       <c r="W19" s="2" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="X19" s="2" t="n">
-        <v>3.69</v>
+        <v>3.5</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>3.56</v>
+        <v>3.44</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>4.06</v>
+        <v>3.96</v>
       </c>
       <c r="AA19" s="2" t="n">
         <v>101.78</v>
@@ -5401,19 +5401,19 @@
         <v>90.92</v>
       </c>
       <c r="V20" s="2" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="W20" s="2" t="n">
-        <v>2.59</v>
+        <v>2.32</v>
       </c>
       <c r="X20" s="2" t="n">
-        <v>2.56</v>
+        <v>2.43</v>
       </c>
       <c r="Y20" s="2" t="n">
-        <v>3.65</v>
+        <v>3.53</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>4.42</v>
+        <v>4.3</v>
       </c>
       <c r="AA20" s="2" t="n">
         <v>107.01</v>
@@ -5647,19 +5647,19 @@
         <v>106.96</v>
       </c>
       <c r="V21" s="2" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="W21" s="2" t="n">
-        <v>11.44</v>
+        <v>10.23</v>
       </c>
       <c r="X21" s="2" t="n">
-        <v>8.960000000000001</v>
+        <v>8.5</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>7.36</v>
+        <v>7.11</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>7.44</v>
+        <v>7.25</v>
       </c>
       <c r="AA21" s="2" t="n">
         <v>101.77</v>
@@ -5893,19 +5893,19 @@
         <v>102.41</v>
       </c>
       <c r="V22" s="2" t="n">
-        <v>0.72</v>
+        <v>0.51</v>
       </c>
       <c r="W22" s="2" t="n">
-        <v>2.19</v>
+        <v>1.96</v>
       </c>
       <c r="X22" s="2" t="n">
-        <v>3.34</v>
+        <v>3.16</v>
       </c>
       <c r="Y22" s="2" t="n">
-        <v>3.88</v>
+        <v>3.75</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>3.79</v>
+        <v>3.69</v>
       </c>
       <c r="AA22" s="2" t="n">
         <v>107.14</v>
@@ -6139,19 +6139,19 @@
         <v>89.73</v>
       </c>
       <c r="V23" s="2" t="n">
-        <v>0.86</v>
+        <v>0.61</v>
       </c>
       <c r="W23" s="2" t="n">
-        <v>2.01</v>
+        <v>1.79</v>
       </c>
       <c r="X23" s="2" t="n">
-        <v>2.23</v>
+        <v>2.12</v>
       </c>
       <c r="Y23" s="2" t="n">
-        <v>4.11</v>
+        <v>3.98</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>3.91</v>
+        <v>3.81</v>
       </c>
       <c r="AA23" s="2" t="n">
         <v>104.24</v>
@@ -6385,19 +6385,19 @@
         <v>85.93000000000001</v>
       </c>
       <c r="V24" s="2" t="n">
-        <v>0.95</v>
+        <v>0.67</v>
       </c>
       <c r="W24" s="2" t="n">
-        <v>0.92</v>
+        <v>0.82</v>
       </c>
       <c r="X24" s="2" t="n">
-        <v>2.81</v>
+        <v>2.67</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>3.36</v>
+        <v>3.25</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>5.28</v>
+        <v>5.15</v>
       </c>
       <c r="AA24" s="2" t="n">
         <v>99.18000000000001</v>
@@ -6631,19 +6631,19 @@
         <v>105.21</v>
       </c>
       <c r="V25" s="2" t="n">
-        <v>2.16</v>
+        <v>1.53</v>
       </c>
       <c r="W25" s="2" t="n">
-        <v>1.72</v>
+        <v>1.54</v>
       </c>
       <c r="X25" s="2" t="n">
-        <v>2.3</v>
+        <v>2.18</v>
       </c>
       <c r="Y25" s="2" t="n">
-        <v>2.66</v>
+        <v>2.57</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>3.25</v>
+        <v>3.17</v>
       </c>
       <c r="AA25" s="2" t="n">
         <v>110.46</v>
@@ -6877,19 +6877,19 @@
         <v>95.28</v>
       </c>
       <c r="V26" s="2" t="n">
-        <v>1.29</v>
+        <v>0.91</v>
       </c>
       <c r="W26" s="2" t="n">
-        <v>2.59</v>
+        <v>2.32</v>
       </c>
       <c r="X26" s="2" t="n">
-        <v>3.34</v>
+        <v>3.17</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>3.01</v>
+        <v>2.91</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>3.66</v>
+        <v>3.57</v>
       </c>
       <c r="AA26" s="2" t="n">
         <v>97.51000000000001</v>
@@ -7123,19 +7123,19 @@
         <v>118.27</v>
       </c>
       <c r="V27" s="2" t="n">
-        <v>0.45</v>
+        <v>0.32</v>
       </c>
       <c r="W27" s="2" t="n">
-        <v>1.02</v>
+        <v>0.92</v>
       </c>
       <c r="X27" s="2" t="n">
-        <v>2.21</v>
+        <v>2.1</v>
       </c>
       <c r="Y27" s="2" t="n">
-        <v>3.93</v>
+        <v>3.8</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>5.1</v>
+        <v>4.97</v>
       </c>
       <c r="AA27" s="2" t="n">
         <v>102.98</v>
@@ -7369,19 +7369,19 @@
         <v>118.98</v>
       </c>
       <c r="V28" s="2" t="n">
-        <v>0.67</v>
+        <v>0.47</v>
       </c>
       <c r="W28" s="2" t="n">
-        <v>1.28</v>
+        <v>1.15</v>
       </c>
       <c r="X28" s="2" t="n">
-        <v>3.84</v>
+        <v>3.64</v>
       </c>
       <c r="Y28" s="2" t="n">
-        <v>6.41</v>
+        <v>6.19</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>7.37</v>
+        <v>7.18</v>
       </c>
       <c r="AA28" s="2" t="n">
         <v>106.15</v>
@@ -7615,19 +7615,19 @@
         <v>111.03</v>
       </c>
       <c r="V29" s="2" t="n">
-        <v>1.1</v>
+        <v>0.78</v>
       </c>
       <c r="W29" s="2" t="n">
-        <v>1.31</v>
+        <v>1.17</v>
       </c>
       <c r="X29" s="2" t="n">
-        <v>2.51</v>
+        <v>2.39</v>
       </c>
       <c r="Y29" s="2" t="n">
-        <v>4.05</v>
+        <v>3.91</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>4.53</v>
+        <v>4.41</v>
       </c>
       <c r="AA29" s="2" t="n">
         <v>98.64</v>
@@ -7861,19 +7861,19 @@
         <v>116.45</v>
       </c>
       <c r="V30" s="2" t="n">
-        <v>1.38</v>
+        <v>0.97</v>
       </c>
       <c r="W30" s="2" t="n">
-        <v>1.62</v>
+        <v>1.45</v>
       </c>
       <c r="X30" s="2" t="n">
-        <v>2.3</v>
+        <v>2.18</v>
       </c>
       <c r="Y30" s="2" t="n">
-        <v>3.58</v>
+        <v>3.46</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>5.03</v>
+        <v>4.91</v>
       </c>
       <c r="AA30" s="2" t="n">
         <v>103.51</v>
@@ -8107,19 +8107,19 @@
         <v>106.97</v>
       </c>
       <c r="V31" s="2" t="n">
-        <v>2.28</v>
+        <v>1.61</v>
       </c>
       <c r="W31" s="2" t="n">
-        <v>3.48</v>
+        <v>3.11</v>
       </c>
       <c r="X31" s="2" t="n">
-        <v>3.43</v>
+        <v>3.26</v>
       </c>
       <c r="Y31" s="2" t="n">
-        <v>3.31</v>
+        <v>3.2</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>3.2</v>
+        <v>3.12</v>
       </c>
       <c r="AA31" s="2" t="n">
         <v>98.22</v>
@@ -8353,19 +8353,19 @@
         <v>96.97</v>
       </c>
       <c r="V32" s="2" t="n">
-        <v>0.48</v>
+        <v>0.34</v>
       </c>
       <c r="W32" s="2" t="n">
-        <v>0.43</v>
+        <v>0.38</v>
       </c>
       <c r="X32" s="2" t="n">
-        <v>1.78</v>
+        <v>1.69</v>
       </c>
       <c r="Y32" s="2" t="n">
-        <v>1.61</v>
+        <v>1.55</v>
       </c>
       <c r="Z32" s="2" t="n">
-        <v>2.32</v>
+        <v>2.27</v>
       </c>
       <c r="AA32" s="2" t="n">
         <v>98.34</v>
@@ -8599,19 +8599,19 @@
         <v>119.62</v>
       </c>
       <c r="V33" s="2" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="W33" s="2" t="n">
-        <v>1.55</v>
+        <v>1.39</v>
       </c>
       <c r="X33" s="2" t="n">
-        <v>5.73</v>
+        <v>5.44</v>
       </c>
       <c r="Y33" s="2" t="n">
-        <v>6.47</v>
+        <v>6.26</v>
       </c>
       <c r="Z33" s="2" t="n">
-        <v>6.89</v>
+        <v>6.72</v>
       </c>
       <c r="AA33" s="2" t="n">
         <v>100.02</v>
@@ -8845,19 +8845,19 @@
         <v>107.57</v>
       </c>
       <c r="V34" s="2" t="n">
-        <v>2.18</v>
+        <v>1.54</v>
       </c>
       <c r="W34" s="2" t="n">
-        <v>2.21</v>
+        <v>1.98</v>
       </c>
       <c r="X34" s="2" t="n">
-        <v>3.39</v>
+        <v>3.21</v>
       </c>
       <c r="Y34" s="2" t="n">
-        <v>4.18</v>
+        <v>4.04</v>
       </c>
       <c r="Z34" s="2" t="n">
-        <v>3.71</v>
+        <v>3.62</v>
       </c>
       <c r="AA34" s="2" t="n">
         <v>100.32</v>
@@ -9091,19 +9091,19 @@
         <v>107.09</v>
       </c>
       <c r="V35" s="2" t="n">
-        <v>3.04</v>
+        <v>2.15</v>
       </c>
       <c r="W35" s="2" t="n">
-        <v>2.41</v>
+        <v>2.15</v>
       </c>
       <c r="X35" s="2" t="n">
-        <v>3.07</v>
+        <v>2.91</v>
       </c>
       <c r="Y35" s="2" t="n">
-        <v>3.07</v>
+        <v>2.97</v>
       </c>
       <c r="Z35" s="2" t="n">
-        <v>2.78</v>
+        <v>2.71</v>
       </c>
       <c r="AA35" s="2" t="n">
         <v>98.48</v>
@@ -9337,19 +9337,19 @@
         <v>113.69</v>
       </c>
       <c r="V36" s="2" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="W36" s="2" t="n">
-        <v>0.79</v>
+        <v>0.71</v>
       </c>
       <c r="X36" s="2" t="n">
-        <v>2.27</v>
+        <v>2.15</v>
       </c>
       <c r="Y36" s="2" t="n">
-        <v>3.98</v>
+        <v>3.84</v>
       </c>
       <c r="Z36" s="2" t="n">
-        <v>4.82</v>
+        <v>4.7</v>
       </c>
       <c r="AA36" s="2" t="n">
         <v>99.03</v>
@@ -9583,19 +9583,19 @@
         <v>105.32</v>
       </c>
       <c r="V37" s="2" t="n">
-        <v>0.66</v>
+        <v>0.47</v>
       </c>
       <c r="W37" s="2" t="n">
-        <v>1.38</v>
+        <v>1.24</v>
       </c>
       <c r="X37" s="2" t="n">
-        <v>1.85</v>
+        <v>1.75</v>
       </c>
       <c r="Y37" s="2" t="n">
-        <v>2.16</v>
+        <v>2.09</v>
       </c>
       <c r="Z37" s="2" t="n">
-        <v>1.94</v>
+        <v>1.9</v>
       </c>
       <c r="AA37" s="2" t="n">
         <v>96.94</v>
@@ -9829,19 +9829,19 @@
         <v>114.7</v>
       </c>
       <c r="V38" s="2" t="n">
-        <v>1.26</v>
+        <v>0.89</v>
       </c>
       <c r="W38" s="2" t="n">
-        <v>2.73</v>
+        <v>2.44</v>
       </c>
       <c r="X38" s="2" t="n">
-        <v>5.88</v>
+        <v>5.58</v>
       </c>
       <c r="Y38" s="2" t="n">
-        <v>6.2</v>
+        <v>5.99</v>
       </c>
       <c r="Z38" s="2" t="n">
-        <v>6.04</v>
+        <v>5.89</v>
       </c>
       <c r="AA38" s="2" t="n">
         <v>99.59999999999999</v>
@@ -10075,19 +10075,19 @@
         <v>106.77</v>
       </c>
       <c r="V39" s="2" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="W39" s="2" t="n">
-        <v>1.76</v>
+        <v>1.57</v>
       </c>
       <c r="X39" s="2" t="n">
-        <v>3.12</v>
+        <v>2.96</v>
       </c>
       <c r="Y39" s="2" t="n">
-        <v>3.68</v>
+        <v>3.55</v>
       </c>
       <c r="Z39" s="2" t="n">
-        <v>3.26</v>
+        <v>3.17</v>
       </c>
       <c r="AA39" s="2" t="n">
         <v>101.67</v>
@@ -10321,19 +10321,19 @@
         <v>123.41</v>
       </c>
       <c r="V40" s="2" t="n">
-        <v>1.15</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="W40" s="2" t="n">
-        <v>1.08</v>
+        <v>0.97</v>
       </c>
       <c r="X40" s="2" t="n">
-        <v>5.03</v>
+        <v>4.77</v>
       </c>
       <c r="Y40" s="2" t="n">
-        <v>6.59</v>
+        <v>6.36</v>
       </c>
       <c r="Z40" s="2" t="n">
-        <v>7.33</v>
+        <v>7.14</v>
       </c>
       <c r="AA40" s="2" t="n">
         <v>106.22</v>
@@ -10567,19 +10567,19 @@
         <v>110.6</v>
       </c>
       <c r="V41" s="2" t="n">
-        <v>0.55</v>
+        <v>0.39</v>
       </c>
       <c r="W41" s="2" t="n">
-        <v>2.01</v>
+        <v>1.8</v>
       </c>
       <c r="X41" s="2" t="n">
-        <v>2.74</v>
+        <v>2.6</v>
       </c>
       <c r="Y41" s="2" t="n">
-        <v>2.58</v>
+        <v>2.49</v>
       </c>
       <c r="Z41" s="2" t="n">
-        <v>2.39</v>
+        <v>2.33</v>
       </c>
       <c r="AA41" s="2" t="n">
         <v>106.39</v>
@@ -10813,19 +10813,19 @@
         <v>118.27</v>
       </c>
       <c r="V42" s="2" t="n">
-        <v>0.45</v>
+        <v>0.32</v>
       </c>
       <c r="W42" s="2" t="n">
-        <v>1.02</v>
+        <v>0.92</v>
       </c>
       <c r="X42" s="2" t="n">
-        <v>2.21</v>
+        <v>2.1</v>
       </c>
       <c r="Y42" s="2" t="n">
-        <v>3.93</v>
+        <v>3.8</v>
       </c>
       <c r="Z42" s="2" t="n">
-        <v>5.1</v>
+        <v>4.97</v>
       </c>
       <c r="AA42" s="2" t="n">
         <v>102.98</v>
@@ -11059,19 +11059,19 @@
         <v>130.13</v>
       </c>
       <c r="V43" s="2" t="n">
-        <v>1.34</v>
+        <v>0.95</v>
       </c>
       <c r="W43" s="2" t="n">
-        <v>1.67</v>
+        <v>1.49</v>
       </c>
       <c r="X43" s="2" t="n">
-        <v>4.17</v>
+        <v>3.96</v>
       </c>
       <c r="Y43" s="2" t="n">
-        <v>6.73</v>
+        <v>6.5</v>
       </c>
       <c r="Z43" s="2" t="n">
-        <v>11.81</v>
+        <v>11.51</v>
       </c>
       <c r="AA43" s="2" t="n">
         <v>107.62</v>
@@ -11305,19 +11305,19 @@
         <v>106.78</v>
       </c>
       <c r="V44" s="2" t="n">
-        <v>0.85</v>
+        <v>0.6</v>
       </c>
       <c r="W44" s="2" t="n">
-        <v>1.19</v>
+        <v>1.07</v>
       </c>
       <c r="X44" s="2" t="n">
-        <v>2.42</v>
+        <v>2.3</v>
       </c>
       <c r="Y44" s="2" t="n">
-        <v>2.31</v>
+        <v>2.23</v>
       </c>
       <c r="Z44" s="2" t="n">
-        <v>2.42</v>
+        <v>2.36</v>
       </c>
       <c r="AA44" s="2" t="n">
         <v>100.18</v>
@@ -11551,19 +11551,19 @@
         <v>100.77</v>
       </c>
       <c r="V45" s="2" t="n">
-        <v>1.12</v>
+        <v>0.79</v>
       </c>
       <c r="W45" s="2" t="n">
-        <v>0.96</v>
+        <v>0.86</v>
       </c>
       <c r="X45" s="2" t="n">
-        <v>1.95</v>
+        <v>1.85</v>
       </c>
       <c r="Y45" s="2" t="n">
-        <v>1.69</v>
+        <v>1.64</v>
       </c>
       <c r="Z45" s="2" t="n">
-        <v>2.12</v>
+        <v>2.06</v>
       </c>
       <c r="AA45" s="2" t="n">
         <v>100.11</v>
@@ -11797,19 +11797,19 @@
         <v>103.49</v>
       </c>
       <c r="V46" s="2" t="n">
-        <v>0.47</v>
+        <v>0.33</v>
       </c>
       <c r="W46" s="2" t="n">
-        <v>1.79</v>
+        <v>1.6</v>
       </c>
       <c r="X46" s="2" t="n">
-        <v>1.73</v>
+        <v>1.64</v>
       </c>
       <c r="Y46" s="2" t="n">
-        <v>2.29</v>
+        <v>2.22</v>
       </c>
       <c r="Z46" s="2" t="n">
-        <v>2.15</v>
+        <v>2.1</v>
       </c>
       <c r="AA46" s="2" t="n">
         <v>101.93</v>

</xml_diff>

<commit_message>
chore: regenerate Excel with correct formatting
- Remove test Excel files
- Regenerate results.xlsx with:
  * Numeric pattern codes (1-8) in column 3
  * All REAL values rounded to 2 decimals
  * Verified: MA200=152.34 (was 152.3357464754)
  * Verified: RSI=7.11 (was 7.1070111972)
</commit_message>
<xml_diff>
--- a/data/results.xlsx
+++ b/data/results.xlsx
@@ -424,90 +424,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CF8"/>
+  <dimension ref="A1:CF9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
-    <col width="20" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="14" max="14"/>
+    <col width="9" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="20" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="20" customWidth="1" min="20" max="20"/>
-    <col width="20" customWidth="1" min="21" max="21"/>
-    <col width="21" customWidth="1" min="22" max="22"/>
-    <col width="20" customWidth="1" min="23" max="23"/>
-    <col width="20" customWidth="1" min="24" max="24"/>
-    <col width="20" customWidth="1" min="25" max="25"/>
-    <col width="20" customWidth="1" min="26" max="26"/>
-    <col width="20" customWidth="1" min="27" max="27"/>
-    <col width="20" customWidth="1" min="28" max="28"/>
-    <col width="20" customWidth="1" min="29" max="29"/>
-    <col width="20" customWidth="1" min="30" max="30"/>
-    <col width="20" customWidth="1" min="31" max="31"/>
-    <col width="20" customWidth="1" min="32" max="32"/>
-    <col width="20" customWidth="1" min="33" max="33"/>
-    <col width="20" customWidth="1" min="34" max="34"/>
-    <col width="20" customWidth="1" min="35" max="35"/>
-    <col width="20" customWidth="1" min="36" max="36"/>
-    <col width="20" customWidth="1" min="37" max="37"/>
-    <col width="20" customWidth="1" min="38" max="38"/>
-    <col width="20" customWidth="1" min="39" max="39"/>
-    <col width="20" customWidth="1" min="40" max="40"/>
-    <col width="20" customWidth="1" min="41" max="41"/>
-    <col width="20" customWidth="1" min="42" max="42"/>
-    <col width="20" customWidth="1" min="43" max="43"/>
-    <col width="20" customWidth="1" min="44" max="44"/>
-    <col width="20" customWidth="1" min="45" max="45"/>
-    <col width="20" customWidth="1" min="46" max="46"/>
-    <col width="20" customWidth="1" min="47" max="47"/>
-    <col width="20" customWidth="1" min="48" max="48"/>
-    <col width="20" customWidth="1" min="49" max="49"/>
-    <col width="20" customWidth="1" min="50" max="50"/>
-    <col width="20" customWidth="1" min="51" max="51"/>
-    <col width="20" customWidth="1" min="52" max="52"/>
-    <col width="20" customWidth="1" min="53" max="53"/>
-    <col width="20" customWidth="1" min="54" max="54"/>
-    <col width="20" customWidth="1" min="55" max="55"/>
-    <col width="20" customWidth="1" min="56" max="56"/>
-    <col width="20" customWidth="1" min="57" max="57"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="8" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="13" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="8" customWidth="1" min="27" max="27"/>
+    <col width="8" customWidth="1" min="28" max="28"/>
+    <col width="8" customWidth="1" min="29" max="29"/>
+    <col width="8" customWidth="1" min="30" max="30"/>
+    <col width="13" customWidth="1" min="31" max="31"/>
+    <col width="13" customWidth="1" min="32" max="32"/>
+    <col width="14" customWidth="1" min="33" max="33"/>
+    <col width="14" customWidth="1" min="34" max="34"/>
+    <col width="14" customWidth="1" min="35" max="35"/>
+    <col width="12" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
+    <col width="12" customWidth="1" min="38" max="38"/>
+    <col width="13" customWidth="1" min="39" max="39"/>
+    <col width="13" customWidth="1" min="40" max="40"/>
+    <col width="16" customWidth="1" min="41" max="41"/>
+    <col width="17" customWidth="1" min="42" max="42"/>
+    <col width="17" customWidth="1" min="43" max="43"/>
+    <col width="16" customWidth="1" min="44" max="44"/>
+    <col width="17" customWidth="1" min="45" max="45"/>
+    <col width="17" customWidth="1" min="46" max="46"/>
+    <col width="17" customWidth="1" min="47" max="47"/>
+    <col width="18" customWidth="1" min="48" max="48"/>
+    <col width="18" customWidth="1" min="49" max="49"/>
+    <col width="17" customWidth="1" min="50" max="50"/>
+    <col width="18" customWidth="1" min="51" max="51"/>
+    <col width="18" customWidth="1" min="52" max="52"/>
+    <col width="17" customWidth="1" min="53" max="53"/>
+    <col width="18" customWidth="1" min="54" max="54"/>
+    <col width="18" customWidth="1" min="55" max="55"/>
+    <col width="16" customWidth="1" min="56" max="56"/>
+    <col width="17" customWidth="1" min="57" max="57"/>
     <col width="7" customWidth="1" min="58" max="58"/>
-    <col width="20" customWidth="1" min="59" max="59"/>
-    <col width="20" customWidth="1" min="60" max="60"/>
-    <col width="19" customWidth="1" min="61" max="61"/>
-    <col width="20" customWidth="1" min="62" max="62"/>
-    <col width="19" customWidth="1" min="63" max="63"/>
-    <col width="20" customWidth="1" min="64" max="64"/>
-    <col width="20" customWidth="1" min="65" max="65"/>
-    <col width="20" customWidth="1" min="66" max="66"/>
-    <col width="20" customWidth="1" min="67" max="67"/>
-    <col width="20" customWidth="1" min="68" max="68"/>
+    <col width="8" customWidth="1" min="59" max="59"/>
+    <col width="8" customWidth="1" min="60" max="60"/>
+    <col width="8" customWidth="1" min="61" max="61"/>
+    <col width="8" customWidth="1" min="62" max="62"/>
+    <col width="8" customWidth="1" min="63" max="63"/>
+    <col width="8" customWidth="1" min="64" max="64"/>
+    <col width="8" customWidth="1" min="65" max="65"/>
+    <col width="8" customWidth="1" min="66" max="66"/>
+    <col width="8" customWidth="1" min="67" max="67"/>
+    <col width="8" customWidth="1" min="68" max="68"/>
     <col width="7" customWidth="1" min="69" max="69"/>
-    <col width="20" customWidth="1" min="70" max="70"/>
-    <col width="20" customWidth="1" min="71" max="71"/>
-    <col width="19" customWidth="1" min="72" max="72"/>
-    <col width="20" customWidth="1" min="73" max="73"/>
-    <col width="19" customWidth="1" min="74" max="74"/>
-    <col width="20" customWidth="1" min="75" max="75"/>
-    <col width="20" customWidth="1" min="76" max="76"/>
-    <col width="20" customWidth="1" min="77" max="77"/>
-    <col width="20" customWidth="1" min="78" max="78"/>
-    <col width="20" customWidth="1" min="79" max="79"/>
-    <col width="20" customWidth="1" min="80" max="80"/>
-    <col width="20" customWidth="1" min="81" max="81"/>
+    <col width="8" customWidth="1" min="70" max="70"/>
+    <col width="8" customWidth="1" min="71" max="71"/>
+    <col width="8" customWidth="1" min="72" max="72"/>
+    <col width="8" customWidth="1" min="73" max="73"/>
+    <col width="8" customWidth="1" min="74" max="74"/>
+    <col width="8" customWidth="1" min="75" max="75"/>
+    <col width="8" customWidth="1" min="76" max="76"/>
+    <col width="8" customWidth="1" min="77" max="77"/>
+    <col width="8" customWidth="1" min="78" max="78"/>
+    <col width="8" customWidth="1" min="79" max="79"/>
+    <col width="10" customWidth="1" min="80" max="80"/>
+    <col width="15" customWidth="1" min="81" max="81"/>
     <col width="20" customWidth="1" min="82" max="82"/>
     <col width="20" customWidth="1" min="83" max="83"/>
     <col width="9" customWidth="1" min="84" max="84"/>
@@ -946,22 +946,20 @@
           <t>2025-10-07</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Hammer</t>
-        </is>
+      <c r="C2" t="n">
+        <v>1</v>
       </c>
       <c r="D2" t="n">
-        <v>0.843</v>
+        <v>0.84</v>
       </c>
       <c r="E2" t="n">
-        <v>102.9367104059533</v>
+        <v>102.94</v>
       </c>
       <c r="F2" t="n">
-        <v>107.2506366198576</v>
+        <v>107.25</v>
       </c>
       <c r="G2" t="n">
-        <v>95.07026740477141</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -970,220 +968,220 @@
         <v>100</v>
       </c>
       <c r="J2" t="n">
-        <v>104.2835477032239</v>
+        <v>104.28</v>
       </c>
       <c r="K2" t="n">
-        <v>29.3143470379756</v>
+        <v>29.31</v>
       </c>
       <c r="L2" t="n">
         <v>1</v>
       </c>
       <c r="M2" t="n">
-        <v>102.6531673383109</v>
+        <v>102.65</v>
       </c>
       <c r="N2" t="n">
-        <v>106.6025282461432</v>
+        <v>106.6</v>
       </c>
       <c r="O2" t="n">
-        <v>10.25626980711295</v>
+        <v>10.26</v>
       </c>
       <c r="P2" t="n">
         <v>1</v>
       </c>
       <c r="Q2" t="n">
-        <v>107.2708863849881</v>
+        <v>107.27</v>
       </c>
       <c r="R2" t="n">
-        <v>110.1772182802611</v>
+        <v>110.18</v>
       </c>
       <c r="S2" t="n">
-        <v>120.8911364591574</v>
+        <v>120.89</v>
       </c>
       <c r="T2" t="n">
-        <v>127.1088573600672</v>
+        <v>127.11</v>
       </c>
       <c r="U2" t="n">
-        <v>137.7316400069225</v>
+        <v>137.73</v>
       </c>
       <c r="V2" t="n">
-        <v>2.111391477947002</v>
+        <v>2.11</v>
       </c>
       <c r="W2" t="n">
-        <v>2.371778464970988</v>
+        <v>2.37</v>
       </c>
       <c r="X2" t="n">
-        <v>4.922886648550141</v>
+        <v>4.92</v>
       </c>
       <c r="Y2" t="n">
-        <v>7.438075216717154</v>
+        <v>7.44</v>
       </c>
       <c r="Z2" t="n">
-        <v>11.26466375241516</v>
+        <v>11.26</v>
       </c>
       <c r="AA2" t="n">
-        <v>105.3670916979826</v>
+        <v>105.37</v>
       </c>
       <c r="AB2" t="n">
-        <v>112.5367060794106</v>
+        <v>112.54</v>
       </c>
       <c r="AC2" t="n">
-        <v>111.4329123195214</v>
+        <v>111.43</v>
       </c>
       <c r="AD2" t="n">
-        <v>84.74936956091771</v>
+        <v>84.75</v>
       </c>
       <c r="AE2" t="n">
-        <v>140.9602170000696</v>
+        <v>140.96</v>
       </c>
       <c r="AF2" t="n">
-        <v>129.6683417294166</v>
+        <v>129.67</v>
       </c>
       <c r="AG2" t="n">
-        <v>126.0502892676559</v>
+        <v>126.05</v>
       </c>
       <c r="AH2" t="n">
-        <v>132.3877657764499</v>
+        <v>132.39</v>
       </c>
       <c r="AI2" t="n">
-        <v>125.9874614335754</v>
+        <v>125.99</v>
       </c>
       <c r="AJ2" t="n">
-        <v>206.3037606352984</v>
+        <v>206.3</v>
       </c>
       <c r="AK2" t="n">
-        <v>147.9907035575093</v>
+        <v>147.99</v>
       </c>
       <c r="AL2" t="n">
-        <v>146.1468883606505</v>
+        <v>146.15</v>
       </c>
       <c r="AM2" t="n">
-        <v>131.1642672664908</v>
+        <v>131.16</v>
       </c>
       <c r="AN2" t="n">
-        <v>175.7027111508501</v>
+        <v>175.7</v>
       </c>
       <c r="AO2" t="n">
-        <v>108.6886079039755</v>
+        <v>108.69</v>
       </c>
       <c r="AP2" t="n">
-        <v>112.6683535032634</v>
+        <v>112.67</v>
       </c>
       <c r="AQ2" t="n">
-        <v>122.3640503702284</v>
+        <v>122.36</v>
       </c>
       <c r="AR2" t="n">
-        <v>112.4516447043117</v>
+        <v>112.45</v>
       </c>
       <c r="AS2" t="n">
-        <v>117.5412651738034</v>
+        <v>117.54</v>
       </c>
       <c r="AT2" t="n">
-        <v>127.368607533129</v>
+        <v>127.37</v>
       </c>
       <c r="AU2" t="n">
-        <v>122.6308856432951</v>
+        <v>122.63</v>
       </c>
       <c r="AV2" t="n">
-        <v>128.3736711333069</v>
+        <v>128.37</v>
       </c>
       <c r="AW2" t="n">
-        <v>135.1782272918315</v>
+        <v>135.18</v>
       </c>
       <c r="AX2" t="n">
-        <v>134.1164566233188</v>
+        <v>134.12</v>
       </c>
       <c r="AY2" t="n">
-        <v>137.1959498924545</v>
+        <v>137.2</v>
       </c>
       <c r="AZ2" t="n">
-        <v>141.9032905675188</v>
+        <v>141.9</v>
       </c>
       <c r="BA2" t="n">
-        <v>140.2754431615902</v>
+        <v>140.28</v>
       </c>
       <c r="BB2" t="n">
-        <v>141.982783450356</v>
+        <v>141.98</v>
       </c>
       <c r="BC2" t="n">
-        <v>145.2182269518889</v>
+        <v>145.22</v>
       </c>
       <c r="BD2" t="n">
-        <v>136.4540756032437</v>
+        <v>136.45</v>
       </c>
       <c r="BE2" t="n">
-        <v>152.3357464754129</v>
+        <v>152.34</v>
       </c>
       <c r="BF2" t="n">
         <v>100</v>
       </c>
       <c r="BG2" t="n">
-        <v>100.0178744396967</v>
+        <v>100.02</v>
       </c>
       <c r="BH2" t="n">
-        <v>99.61084915950865</v>
+        <v>99.61</v>
       </c>
       <c r="BI2" t="n">
-        <v>99.14112517343587</v>
+        <v>99.14</v>
       </c>
       <c r="BJ2" t="n">
-        <v>98.39409285400554</v>
+        <v>98.39</v>
       </c>
       <c r="BK2" t="n">
-        <v>96.99192377838604</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="BL2" t="n">
-        <v>100.3056034695902</v>
+        <v>100.31</v>
       </c>
       <c r="BM2" t="n">
-        <v>98.95332720550806</v>
+        <v>98.95</v>
       </c>
       <c r="BN2" t="n">
-        <v>100.3091812663073</v>
+        <v>100.31</v>
       </c>
       <c r="BO2" t="n">
-        <v>102.625630113995</v>
+        <v>102.63</v>
       </c>
       <c r="BP2" t="n">
-        <v>100.8483014191927</v>
+        <v>100.85</v>
       </c>
       <c r="BQ2" t="n">
         <v>100</v>
       </c>
       <c r="BR2" t="n">
-        <v>99.77974867194236</v>
+        <v>99.78</v>
       </c>
       <c r="BS2" t="n">
-        <v>99.35491647480248</v>
+        <v>99.34999999999999</v>
       </c>
       <c r="BT2" t="n">
-        <v>98.95306709330993</v>
+        <v>98.95</v>
       </c>
       <c r="BU2" t="n">
-        <v>97.72151683752682</v>
+        <v>97.72</v>
       </c>
       <c r="BV2" t="n">
-        <v>95.97254265108941</v>
+        <v>95.97</v>
       </c>
       <c r="BW2" t="n">
-        <v>101.0384332749026</v>
+        <v>101.04</v>
       </c>
       <c r="BX2" t="n">
-        <v>98.94964679744724</v>
+        <v>98.95</v>
       </c>
       <c r="BY2" t="n">
-        <v>101.154982804954</v>
+        <v>101.15</v>
       </c>
       <c r="BZ2" t="n">
-        <v>104.7178303089793</v>
+        <v>104.72</v>
       </c>
       <c r="CA2" t="n">
-        <v>102.3971949485297</v>
+        <v>102.4</v>
       </c>
       <c r="CB2" t="n">
-        <v>7.10701119722178</v>
+        <v>7.11</v>
       </c>
       <c r="CC2" t="n">
-        <v>104.1417684434335</v>
+        <v>104.14</v>
       </c>
       <c r="CD2" t="n">
         <v>0</v>
@@ -1206,22 +1204,20 @@
           <t>2025-10-03</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Piercing Pattern</t>
-        </is>
+      <c r="C3" t="n">
+        <v>3</v>
       </c>
       <c r="D3" t="n">
         <v>0.55</v>
       </c>
       <c r="E3" t="n">
-        <v>101.9628926819132</v>
+        <v>101.96</v>
       </c>
       <c r="F3" t="n">
-        <v>104.0917917476327</v>
+        <v>104.09</v>
       </c>
       <c r="G3" t="n">
-        <v>39.44970182266147</v>
+        <v>39.45</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -1230,220 +1226,220 @@
         <v>100</v>
       </c>
       <c r="J3" t="n">
-        <v>103.7988274723466</v>
+        <v>103.8</v>
       </c>
       <c r="K3" t="n">
-        <v>20.56563437739031</v>
+        <v>20.57</v>
       </c>
       <c r="L3" t="n">
         <v>1</v>
       </c>
       <c r="M3" t="n">
-        <v>99.26757813591394</v>
+        <v>99.27</v>
       </c>
       <c r="N3" t="n">
-        <v>103.4277364100853</v>
+        <v>103.43</v>
       </c>
       <c r="O3" t="n">
-        <v>95.07026740477141</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="P3" t="n">
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>104.6484395168954</v>
+        <v>104.65</v>
       </c>
       <c r="R3" t="n">
-        <v>107.3046832188266</v>
+        <v>107.3</v>
       </c>
       <c r="S3" t="n">
-        <v>117.5878924490825</v>
+        <v>117.59</v>
       </c>
       <c r="T3" t="n">
-        <v>132.7929625989055</v>
+        <v>132.79</v>
       </c>
       <c r="U3" t="n">
-        <v>135.576171642897</v>
+        <v>135.58</v>
       </c>
       <c r="V3" t="n">
-        <v>0.9033232792716746</v>
+        <v>0.9</v>
       </c>
       <c r="W3" t="n">
-        <v>1.642634594693139</v>
+        <v>1.64</v>
       </c>
       <c r="X3" t="n">
-        <v>5.182260403457925</v>
+        <v>5.18</v>
       </c>
       <c r="Y3" t="n">
-        <v>8.394641164995759</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="Z3" t="n">
-        <v>11.07531739755949</v>
+        <v>11.08</v>
       </c>
       <c r="AA3" t="n">
-        <v>100.4296824272024</v>
+        <v>100.43</v>
       </c>
       <c r="AB3" t="n">
-        <v>100.3320276687737</v>
+        <v>100.33</v>
       </c>
       <c r="AC3" t="n">
-        <v>109.1601534312941</v>
+        <v>109.16</v>
       </c>
       <c r="AD3" t="n">
-        <v>77.10937295691113</v>
+        <v>77.11</v>
       </c>
       <c r="AE3" t="n">
-        <v>114.5775656125489</v>
+        <v>114.58</v>
       </c>
       <c r="AF3" t="n">
-        <v>123.9268780741626</v>
+        <v>123.93</v>
       </c>
       <c r="AG3" t="n">
-        <v>127.8387613777254</v>
+        <v>127.84</v>
       </c>
       <c r="AH3" t="n">
-        <v>128.2480414514688</v>
+        <v>128.25</v>
       </c>
       <c r="AI3" t="n">
-        <v>118.5676552996295</v>
+        <v>118.57</v>
       </c>
       <c r="AJ3" t="n">
-        <v>149.8330033023949</v>
+        <v>149.83</v>
       </c>
       <c r="AK3" t="n">
-        <v>170.2005524498932</v>
+        <v>170.2</v>
       </c>
       <c r="AL3" t="n">
-        <v>148.5212215628555</v>
+        <v>148.52</v>
       </c>
       <c r="AM3" t="n">
-        <v>146.2610570791897</v>
+        <v>146.26</v>
       </c>
       <c r="AN3" t="n">
-        <v>168.5670817861504</v>
+        <v>168.57</v>
       </c>
       <c r="AO3" t="n">
-        <v>106.7675768320623</v>
+        <v>106.77</v>
       </c>
       <c r="AP3" t="n">
-        <v>111.7695292566787</v>
+        <v>111.77</v>
       </c>
       <c r="AQ3" t="n">
-        <v>121.3061508341707</v>
+        <v>121.31</v>
       </c>
       <c r="AR3" t="n">
-        <v>112.4902306126024</v>
+        <v>112.49</v>
       </c>
       <c r="AS3" t="n">
-        <v>116.8818337189878</v>
+        <v>116.88</v>
       </c>
       <c r="AT3" t="n">
-        <v>125.8037086456461</v>
+        <v>125.8</v>
       </c>
       <c r="AU3" t="n">
-        <v>121.2734368253732</v>
+        <v>121.27</v>
       </c>
       <c r="AV3" t="n">
-        <v>127.3525375522295</v>
+        <v>127.35</v>
       </c>
       <c r="AW3" t="n">
-        <v>132.9291968356193</v>
+        <v>132.93</v>
       </c>
       <c r="AX3" t="n">
-        <v>133.4316382790858</v>
+        <v>133.43</v>
       </c>
       <c r="AY3" t="n">
-        <v>134.7255835723045</v>
+        <v>134.73</v>
       </c>
       <c r="AZ3" t="n">
-        <v>138.5957004339144</v>
+        <v>138.6</v>
       </c>
       <c r="BA3" t="n">
-        <v>136.0195288655232</v>
+        <v>136.02</v>
       </c>
       <c r="BB3" t="n">
-        <v>138.505856119009</v>
+        <v>138.51</v>
       </c>
       <c r="BC3" t="n">
-        <v>141.1337868700357</v>
+        <v>141.13</v>
       </c>
       <c r="BD3" t="n">
-        <v>133.8572245261487</v>
+        <v>133.86</v>
       </c>
       <c r="BE3" t="n">
-        <v>147.2813939708263</v>
+        <v>147.28</v>
       </c>
       <c r="BF3" t="n">
         <v>100</v>
       </c>
       <c r="BG3" t="n">
-        <v>99.93165593737589</v>
+        <v>99.93000000000001</v>
       </c>
       <c r="BH3" t="n">
-        <v>98.92656197810402</v>
+        <v>98.93000000000001</v>
       </c>
       <c r="BI3" t="n">
-        <v>99.23419023700703</v>
+        <v>99.23</v>
       </c>
       <c r="BJ3" t="n">
-        <v>98.0419280645296</v>
+        <v>98.04000000000001</v>
       </c>
       <c r="BK3" t="n">
-        <v>96.51135551141789</v>
+        <v>96.51000000000001</v>
       </c>
       <c r="BL3" t="n">
-        <v>99.98212875468829</v>
+        <v>99.98</v>
       </c>
       <c r="BM3" t="n">
-        <v>97.56871086666233</v>
+        <v>97.56999999999999</v>
       </c>
       <c r="BN3" t="n">
-        <v>99.2289771845707</v>
+        <v>99.23</v>
       </c>
       <c r="BO3" t="n">
-        <v>101.1301708645189</v>
+        <v>101.13</v>
       </c>
       <c r="BP3" t="n">
-        <v>101.8525021706511</v>
+        <v>101.85</v>
       </c>
       <c r="BQ3" t="n">
         <v>100</v>
       </c>
       <c r="BR3" t="n">
-        <v>100.0618903458153</v>
+        <v>100.06</v>
       </c>
       <c r="BS3" t="n">
-        <v>98.86357063639572</v>
+        <v>98.86</v>
       </c>
       <c r="BT3" t="n">
-        <v>99.35740894577904</v>
+        <v>99.36</v>
       </c>
       <c r="BU3" t="n">
-        <v>97.20268087481145</v>
+        <v>97.2</v>
       </c>
       <c r="BV3" t="n">
-        <v>95.42845944102001</v>
+        <v>95.43000000000001</v>
       </c>
       <c r="BW3" t="n">
-        <v>100.2207375053447</v>
+        <v>100.22</v>
       </c>
       <c r="BX3" t="n">
-        <v>97.72536824913362</v>
+        <v>97.73</v>
       </c>
       <c r="BY3" t="n">
-        <v>100.1308412658412</v>
+        <v>100.13</v>
       </c>
       <c r="BZ3" t="n">
-        <v>102.310383787913</v>
+        <v>102.31</v>
       </c>
       <c r="CA3" t="n">
-        <v>104.3275725036654</v>
+        <v>104.33</v>
       </c>
       <c r="CB3" t="n">
-        <v>2.563052866730388</v>
+        <v>2.56</v>
       </c>
       <c r="CC3" t="n">
-        <v>103.4472643815389</v>
+        <v>103.45</v>
       </c>
       <c r="CD3" t="n">
         <v>0</v>
@@ -1463,25 +1459,23 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025-09-23</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Hammer</t>
-        </is>
+          <t>2025-10-03</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1</v>
       </c>
       <c r="D4" t="n">
-        <v>0.858</v>
+        <v>0.99</v>
       </c>
       <c r="E4" t="n">
-        <v>100.9643849069264</v>
+        <v>101.96</v>
       </c>
       <c r="F4" t="n">
-        <v>102.4025073930131</v>
+        <v>104.09</v>
       </c>
       <c r="G4" t="n">
-        <v>27.64705618360762</v>
+        <v>39.45</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -1490,220 +1484,220 @@
         <v>100</v>
       </c>
       <c r="J4" t="n">
-        <v>101.497338876719</v>
+        <v>103.8</v>
       </c>
       <c r="K4" t="n">
-        <v>28.24851938378779</v>
+        <v>20.57</v>
       </c>
       <c r="L4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="n">
-        <v>97.77514823298613</v>
+        <v>99.27</v>
       </c>
       <c r="N4" t="n">
-        <v>101.4381224860867</v>
+        <v>103.43</v>
       </c>
       <c r="O4" t="n">
-        <v>79.44575027046457</v>
+        <v>95.06999999999999</v>
       </c>
       <c r="P4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>101.8610985489177</v>
+        <v>104.65</v>
       </c>
       <c r="R4" t="n">
-        <v>106.1839079732756</v>
+        <v>107.3</v>
       </c>
       <c r="S4" t="n">
-        <v>115.0579439643202</v>
+        <v>117.59</v>
       </c>
       <c r="T4" t="n">
-        <v>117.2828021854366</v>
+        <v>132.79</v>
       </c>
       <c r="U4" t="n">
-        <v>122.9253013146168</v>
+        <v>135.58</v>
       </c>
       <c r="V4" t="n">
-        <v>0.3468434694905866</v>
+        <v>0.9</v>
       </c>
       <c r="W4" t="n">
-        <v>1.798809566283605</v>
+        <v>1.64</v>
       </c>
       <c r="X4" t="n">
-        <v>5.624250393803055</v>
+        <v>5.18</v>
       </c>
       <c r="Y4" t="n">
-        <v>6.252945465636911</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="Z4" t="n">
-        <v>6.853142939175644</v>
+        <v>11.08</v>
       </c>
       <c r="AA4" t="n">
-        <v>94.20522923003654</v>
+        <v>100.43</v>
       </c>
       <c r="AB4" t="n">
-        <v>92.03959385365491</v>
+        <v>100.33</v>
       </c>
       <c r="AC4" t="n">
-        <v>86.99771350509981</v>
+        <v>109.16</v>
       </c>
       <c r="AD4" t="n">
-        <v>93.08857268232694</v>
+        <v>77.11</v>
       </c>
       <c r="AE4" t="n">
-        <v>148.9968125765601</v>
+        <v>114.58</v>
       </c>
       <c r="AF4" t="n">
-        <v>146.7517486705061</v>
+        <v>123.93</v>
       </c>
       <c r="AG4" t="n">
-        <v>127.390830221901</v>
+        <v>127.84</v>
       </c>
       <c r="AH4" t="n">
-        <v>112.2654519298585</v>
+        <v>128.25</v>
       </c>
       <c r="AI4" t="n">
-        <v>103.3512069976236</v>
+        <v>118.57</v>
       </c>
       <c r="AJ4" t="n">
-        <v>121.9289269708131</v>
+        <v>149.83</v>
       </c>
       <c r="AK4" t="n">
-        <v>121.8842778290222</v>
+        <v>170.2</v>
       </c>
       <c r="AL4" t="n">
-        <v>127.4349540796709</v>
+        <v>148.52</v>
       </c>
       <c r="AM4" t="n">
-        <v>136.1956409830796</v>
+        <v>146.26</v>
       </c>
       <c r="AN4" t="n">
-        <v>134.4435561307999</v>
+        <v>168.57</v>
       </c>
       <c r="AO4" t="n">
-        <v>105.05371975422</v>
+        <v>106.77</v>
       </c>
       <c r="AP4" t="n">
-        <v>110.3197710910551</v>
+        <v>111.77</v>
       </c>
       <c r="AQ4" t="n">
-        <v>115.1505800205124</v>
+        <v>121.31</v>
       </c>
       <c r="AR4" t="n">
-        <v>112.0379002971533</v>
+        <v>112.49</v>
       </c>
       <c r="AS4" t="n">
-        <v>114.6104403756778</v>
+        <v>116.88</v>
       </c>
       <c r="AT4" t="n">
-        <v>118.5428479153346</v>
+        <v>125.8</v>
       </c>
       <c r="AU4" t="n">
-        <v>117.1829804542023</v>
+        <v>121.27</v>
       </c>
       <c r="AV4" t="n">
-        <v>118.6092544988806</v>
+        <v>127.35</v>
       </c>
       <c r="AW4" t="n">
-        <v>121.3120719276165</v>
+        <v>132.93</v>
       </c>
       <c r="AX4" t="n">
-        <v>120.0355285435588</v>
+        <v>133.43</v>
       </c>
       <c r="AY4" t="n">
-        <v>122.4752554549913</v>
+        <v>134.73</v>
       </c>
       <c r="AZ4" t="n">
-        <v>123.6976573092291</v>
+        <v>138.6</v>
       </c>
       <c r="BA4" t="n">
-        <v>124.9149823664238</v>
+        <v>136.02</v>
       </c>
       <c r="BB4" t="n">
-        <v>124.0148893563524</v>
+        <v>138.51</v>
       </c>
       <c r="BC4" t="n">
-        <v>126.4453100973595</v>
+        <v>141.13</v>
       </c>
       <c r="BD4" t="n">
-        <v>123.6015572716727</v>
+        <v>133.86</v>
       </c>
       <c r="BE4" t="n">
-        <v>128.9389229884224</v>
+        <v>147.28</v>
       </c>
       <c r="BF4" t="n">
         <v>100</v>
       </c>
       <c r="BG4" t="n">
-        <v>100.1117625192066</v>
+        <v>99.93000000000001</v>
       </c>
       <c r="BH4" t="n">
-        <v>99.24649602460785</v>
+        <v>98.93000000000001</v>
       </c>
       <c r="BI4" t="n">
-        <v>97.8321797424731</v>
+        <v>99.23</v>
       </c>
       <c r="BJ4" t="n">
-        <v>96.37400050405725</v>
+        <v>98.04000000000001</v>
       </c>
       <c r="BK4" t="n">
-        <v>96.73121953981743</v>
+        <v>96.51000000000001</v>
       </c>
       <c r="BL4" t="n">
-        <v>99.21585796969377</v>
+        <v>99.98</v>
       </c>
       <c r="BM4" t="n">
-        <v>100.4737932772611</v>
+        <v>97.56999999999999</v>
       </c>
       <c r="BN4" t="n">
-        <v>100.8663153913793</v>
+        <v>99.23</v>
       </c>
       <c r="BO4" t="n">
-        <v>99.81057510937133</v>
+        <v>101.13</v>
       </c>
       <c r="BP4" t="n">
-        <v>101.1781751425839</v>
+        <v>101.85</v>
       </c>
       <c r="BQ4" t="n">
         <v>100</v>
       </c>
       <c r="BR4" t="n">
-        <v>100.1874685092555</v>
+        <v>100.06</v>
       </c>
       <c r="BS4" t="n">
-        <v>98.75541982481273</v>
+        <v>98.86</v>
       </c>
       <c r="BT4" t="n">
-        <v>96.98794132433514</v>
+        <v>99.36</v>
       </c>
       <c r="BU4" t="n">
-        <v>94.51158982560813</v>
+        <v>97.2</v>
       </c>
       <c r="BV4" t="n">
-        <v>95.30287809016525</v>
+        <v>95.43000000000001</v>
       </c>
       <c r="BW4" t="n">
-        <v>99.25606952441258</v>
+        <v>100.22</v>
       </c>
       <c r="BX4" t="n">
-        <v>100.4061009863531</v>
+        <v>97.73</v>
       </c>
       <c r="BY4" t="n">
-        <v>101.0580095568972</v>
+        <v>100.13</v>
       </c>
       <c r="BZ4" t="n">
-        <v>99.99654351708023</v>
+        <v>102.31</v>
       </c>
       <c r="CA4" t="n">
-        <v>102.2252121903081</v>
+        <v>104.33</v>
       </c>
       <c r="CB4" t="n">
-        <v>19.14063538036321</v>
+        <v>2.56</v>
       </c>
       <c r="CC4" t="n">
-        <v>100.9897624380398</v>
+        <v>103.45</v>
       </c>
       <c r="CD4" t="n">
         <v>0</v>
@@ -1712,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="CF4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -1723,247 +1717,245 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2025-09-03</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Hammer</t>
-        </is>
+          <t>2025-09-23</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>0.99</v>
+        <v>0.86</v>
       </c>
       <c r="E5" t="n">
-        <v>100.858210337586</v>
+        <v>100.96</v>
       </c>
       <c r="F5" t="n">
-        <v>102.6919959800876</v>
+        <v>102.4</v>
       </c>
       <c r="G5" t="n">
-        <v>7.60009765625</v>
+        <v>27.65</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
         <v>100</v>
       </c>
       <c r="J5" t="n">
-        <v>101.6724116105583</v>
+        <v>101.5</v>
       </c>
       <c r="K5" t="n">
-        <v>17.10524554617125</v>
+        <v>28.25</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>101.701747256121</v>
+        <v>97.78</v>
       </c>
       <c r="N5" t="n">
-        <v>103.4768616074971</v>
+        <v>101.44</v>
       </c>
       <c r="O5" t="n">
-        <v>44.21493335351013</v>
+        <v>79.45</v>
       </c>
       <c r="P5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>103.0880887541506</v>
+        <v>101.86</v>
       </c>
       <c r="R5" t="n">
-        <v>105.8314361046471</v>
+        <v>106.18</v>
       </c>
       <c r="S5" t="n">
-        <v>108.0099743433421</v>
+        <v>115.06</v>
       </c>
       <c r="T5" t="n">
-        <v>108.4354139555072</v>
+        <v>117.28</v>
       </c>
       <c r="U5" t="n">
-        <v>109.4696717440875</v>
+        <v>122.93</v>
       </c>
       <c r="V5" t="n">
-        <v>0.6968363056427194</v>
+        <v>0.35</v>
       </c>
       <c r="W5" t="n">
-        <v>1.660009965424125</v>
+        <v>1.8</v>
       </c>
       <c r="X5" t="n">
-        <v>2.629421272998699</v>
+        <v>5.62</v>
       </c>
       <c r="Y5" t="n">
-        <v>2.252660837951285</v>
+        <v>6.25</v>
       </c>
       <c r="Z5" t="n">
-        <v>2.498697471945422</v>
+        <v>6.85</v>
       </c>
       <c r="AA5" t="n">
-        <v>101.8337856425016</v>
+        <v>94.20999999999999</v>
       </c>
       <c r="AB5" t="n">
-        <v>98.36426634079962</v>
+        <v>92.04000000000001</v>
       </c>
       <c r="AC5" t="n">
-        <v>90.48631919129873</v>
+        <v>87</v>
       </c>
       <c r="AD5" t="n">
-        <v>78.60339046639648</v>
+        <v>93.09</v>
       </c>
       <c r="AE5" t="n">
-        <v>97.51903384547276</v>
+        <v>149</v>
       </c>
       <c r="AF5" t="n">
-        <v>89.92091325015541</v>
+        <v>146.75</v>
       </c>
       <c r="AG5" t="n">
-        <v>87.93039176656443</v>
+        <v>127.39</v>
       </c>
       <c r="AH5" t="n">
-        <v>90.85147516087983</v>
+        <v>112.27</v>
       </c>
       <c r="AI5" t="n">
-        <v>86.79554673816025</v>
+        <v>103.35</v>
       </c>
       <c r="AJ5" t="n">
-        <v>84.53797050504183</v>
+        <v>121.93</v>
       </c>
       <c r="AK5" t="n">
-        <v>86.50921999639888</v>
+        <v>121.88</v>
       </c>
       <c r="AL5" t="n">
-        <v>93.27754366895783</v>
+        <v>127.43</v>
       </c>
       <c r="AM5" t="n">
-        <v>111.0110802942778</v>
+        <v>136.2</v>
       </c>
       <c r="AN5" t="n">
-        <v>124.9023322965001</v>
+        <v>134.44</v>
       </c>
       <c r="AO5" t="n">
-        <v>105.0597776736374</v>
+        <v>105.05</v>
       </c>
       <c r="AP5" t="n">
-        <v>106.634633992212</v>
+        <v>110.32</v>
       </c>
       <c r="AQ5" t="n">
-        <v>107.8130253847911</v>
+        <v>115.15</v>
       </c>
       <c r="AR5" t="n">
-        <v>107.8764742113261</v>
+        <v>112.04</v>
       </c>
       <c r="AS5" t="n">
-        <v>107.2713249493006</v>
+        <v>114.61</v>
       </c>
       <c r="AT5" t="n">
-        <v>109.1747947819934</v>
+        <v>118.54</v>
       </c>
       <c r="AU5" t="n">
-        <v>106.6661756872751</v>
+        <v>117.18</v>
       </c>
       <c r="AV5" t="n">
-        <v>108.1706141447059</v>
+        <v>118.61</v>
       </c>
       <c r="AW5" t="n">
-        <v>111.7424617967853</v>
+        <v>121.31</v>
       </c>
       <c r="AX5" t="n">
-        <v>109.6750526021367</v>
+        <v>120.04</v>
       </c>
       <c r="AY5" t="n">
-        <v>111.0782646146862</v>
+        <v>122.48</v>
       </c>
       <c r="AZ5" t="n">
-        <v>115.6348553806398</v>
+        <v>123.7</v>
       </c>
       <c r="BA5" t="n">
-        <v>112.4814766272357</v>
+        <v>124.91</v>
       </c>
       <c r="BB5" t="n">
-        <v>115.3143094488648</v>
+        <v>124.01</v>
       </c>
       <c r="BC5" t="n">
-        <v>117.826595219465</v>
+        <v>126.45</v>
       </c>
       <c r="BD5" t="n">
-        <v>113.7222895950909</v>
+        <v>123.6</v>
       </c>
       <c r="BE5" t="n">
-        <v>112.6731809017672</v>
+        <v>128.94</v>
       </c>
       <c r="BF5" t="n">
         <v>100</v>
       </c>
       <c r="BG5" t="n">
-        <v>100.1860967212266</v>
+        <v>100.11</v>
       </c>
       <c r="BH5" t="n">
-        <v>100.2741852286333</v>
+        <v>99.25</v>
       </c>
       <c r="BI5" t="n">
-        <v>99.4279131148817</v>
+        <v>97.83</v>
       </c>
       <c r="BJ5" t="n">
-        <v>99.96122984974447</v>
+        <v>96.37</v>
       </c>
       <c r="BK5" t="n">
-        <v>97.68821620658917</v>
+        <v>96.73</v>
       </c>
       <c r="BL5" t="n">
-        <v>100.5154915524992</v>
+        <v>99.22</v>
       </c>
       <c r="BM5" t="n">
-        <v>101.2992695158487</v>
+        <v>100.47</v>
       </c>
       <c r="BN5" t="n">
-        <v>102.3586260101063</v>
+        <v>100.87</v>
       </c>
       <c r="BO5" t="n">
-        <v>102.9420410485024</v>
+        <v>99.81</v>
       </c>
       <c r="BP5" t="n">
-        <v>104.0776959868957</v>
+        <v>101.18</v>
       </c>
       <c r="BQ5" t="n">
         <v>100</v>
       </c>
       <c r="BR5" t="n">
-        <v>100.0024773952283</v>
+        <v>100.19</v>
       </c>
       <c r="BS5" t="n">
-        <v>100.4717060611434</v>
+        <v>98.76000000000001</v>
       </c>
       <c r="BT5" t="n">
-        <v>99.8715758352367</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="BU5" t="n">
-        <v>101.8123522425598</v>
+        <v>94.51000000000001</v>
       </c>
       <c r="BV5" t="n">
-        <v>98.30757203756498</v>
+        <v>95.3</v>
       </c>
       <c r="BW5" t="n">
-        <v>101.0147394172266</v>
+        <v>99.26000000000001</v>
       </c>
       <c r="BX5" t="n">
-        <v>101.8553604910347</v>
+        <v>100.41</v>
       </c>
       <c r="BY5" t="n">
-        <v>103.4544315262139</v>
+        <v>101.06</v>
       </c>
       <c r="BZ5" t="n">
-        <v>104.6497455289689</v>
+        <v>100</v>
       </c>
       <c r="CA5" t="n">
-        <v>105.9194064127667</v>
+        <v>102.23</v>
       </c>
       <c r="CB5" t="n">
-        <v>34.81796401948304</v>
+        <v>19.14</v>
       </c>
       <c r="CC5" t="n">
-        <v>101.4743596272571</v>
+        <v>100.99</v>
       </c>
       <c r="CD5" t="n">
         <v>0</v>
@@ -1972,7 +1964,7 @@
         <v>0</v>
       </c>
       <c r="CF5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -1983,247 +1975,245 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025-08-13</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Hammer</t>
-        </is>
+          <t>2025-09-03</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>1</v>
       </c>
       <c r="D6" t="n">
-        <v>0.736</v>
+        <v>0.99</v>
       </c>
       <c r="E6" t="n">
-        <v>102.3969559669065</v>
+        <v>100.86</v>
       </c>
       <c r="F6" t="n">
-        <v>105.3736876879702</v>
+        <v>102.69</v>
       </c>
       <c r="G6" t="n">
-        <v>5.225692808420259</v>
+        <v>7.6</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
         <v>100</v>
       </c>
       <c r="J6" t="n">
-        <v>104.0302711604448</v>
+        <v>101.67</v>
       </c>
       <c r="K6" t="n">
-        <v>27.71900330874086</v>
+        <v>17.11</v>
       </c>
       <c r="L6" t="n">
         <v>1</v>
       </c>
       <c r="M6" t="n">
-        <v>101.2161502579203</v>
+        <v>101.7</v>
       </c>
       <c r="N6" t="n">
-        <v>105.4231873187729</v>
+        <v>103.48</v>
       </c>
       <c r="O6" t="n">
-        <v>62.52090065138226</v>
+        <v>44.21</v>
       </c>
       <c r="P6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" t="n">
-        <v>105.1686439906283</v>
+        <v>103.09</v>
       </c>
       <c r="R6" t="n">
-        <v>106.5898379458905</v>
+        <v>105.83</v>
       </c>
       <c r="S6" t="n">
-        <v>111.7584711475844</v>
+        <v>108.01</v>
       </c>
       <c r="T6" t="n">
-        <v>115.491766101082</v>
+        <v>108.44</v>
       </c>
       <c r="U6" t="n">
-        <v>118.2705316657381</v>
+        <v>109.47</v>
       </c>
       <c r="V6" t="n">
-        <v>0.3217152334142881</v>
+        <v>0.7</v>
       </c>
       <c r="W6" t="n">
-        <v>0.9159765755472358</v>
+        <v>1.66</v>
       </c>
       <c r="X6" t="n">
-        <v>2.098484276469901</v>
+        <v>2.63</v>
       </c>
       <c r="Y6" t="n">
-        <v>3.799397856748029</v>
+        <v>2.25</v>
       </c>
       <c r="Z6" t="n">
-        <v>4.969716504903118</v>
+        <v>2.5</v>
       </c>
       <c r="AA6" t="n">
-        <v>102.9767425099981</v>
+        <v>101.83</v>
       </c>
       <c r="AB6" t="n">
-        <v>106.8090259361666</v>
+        <v>98.36</v>
       </c>
       <c r="AC6" t="n">
-        <v>102.2343235704986</v>
+        <v>90.48999999999999</v>
       </c>
       <c r="AD6" t="n">
-        <v>97.3768000797518</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="AE6" t="n">
-        <v>75.50277444531552</v>
+        <v>97.52</v>
       </c>
       <c r="AF6" t="n">
-        <v>74.4307490702294</v>
+        <v>89.92</v>
       </c>
       <c r="AG6" t="n">
-        <v>103.7616906685783</v>
+        <v>87.93000000000001</v>
       </c>
       <c r="AH6" t="n">
-        <v>89.11467798230821</v>
+        <v>90.84999999999999</v>
       </c>
       <c r="AI6" t="n">
-        <v>81.97338867493845</v>
+        <v>86.8</v>
       </c>
       <c r="AJ6" t="n">
-        <v>165.4628885546425</v>
+        <v>84.54000000000001</v>
       </c>
       <c r="AK6" t="n">
-        <v>80.71560012416946</v>
+        <v>86.51000000000001</v>
       </c>
       <c r="AL6" t="n">
-        <v>83.8067430123313</v>
+        <v>93.28</v>
       </c>
       <c r="AM6" t="n">
-        <v>80.55902440780828</v>
+        <v>111.01</v>
       </c>
       <c r="AN6" t="n">
-        <v>87.43608082798548</v>
+        <v>124.9</v>
       </c>
       <c r="AO6" t="n">
-        <v>105.9195430325278</v>
+        <v>105.06</v>
       </c>
       <c r="AP6" t="n">
-        <v>107.7168974995134</v>
+        <v>106.63</v>
       </c>
       <c r="AQ6" t="n">
-        <v>112.0596820112645</v>
+        <v>107.81</v>
       </c>
       <c r="AR6" t="n">
-        <v>107.3916478112057</v>
+        <v>107.88</v>
       </c>
       <c r="AS6" t="n">
-        <v>110.2658619991723</v>
+        <v>107.27</v>
       </c>
       <c r="AT6" t="n">
-        <v>113.2595684900973</v>
+        <v>109.17</v>
       </c>
       <c r="AU6" t="n">
-        <v>113.1400761871388</v>
+        <v>106.67</v>
       </c>
       <c r="AV6" t="n">
-        <v>115.206115038523</v>
+        <v>108.17</v>
       </c>
       <c r="AW6" t="n">
-        <v>114.8713198405482</v>
+        <v>111.74</v>
       </c>
       <c r="AX6" t="n">
-        <v>117.2721538899071</v>
+        <v>109.68</v>
       </c>
       <c r="AY6" t="n">
-        <v>116.2532749810223</v>
+        <v>111.08</v>
       </c>
       <c r="AZ6" t="n">
-        <v>115.3613149380564</v>
+        <v>115.63</v>
       </c>
       <c r="BA6" t="n">
-        <v>115.2343960721374</v>
+        <v>112.48</v>
       </c>
       <c r="BB6" t="n">
-        <v>114.5365246425734</v>
+        <v>115.31</v>
       </c>
       <c r="BC6" t="n">
-        <v>115.3436388874623</v>
+        <v>117.83</v>
       </c>
       <c r="BD6" t="n">
-        <v>113.7112410770118</v>
+        <v>113.72</v>
       </c>
       <c r="BE6" t="n">
-        <v>107.9836721076701</v>
+        <v>112.67</v>
       </c>
       <c r="BF6" t="n">
         <v>100</v>
       </c>
       <c r="BG6" t="n">
-        <v>98.55982788912586</v>
+        <v>100.19</v>
       </c>
       <c r="BH6" t="n">
-        <v>98.12079927777705</v>
+        <v>100.27</v>
       </c>
       <c r="BI6" t="n">
-        <v>98.39667684419501</v>
+        <v>99.43000000000001</v>
       </c>
       <c r="BJ6" t="n">
-        <v>98.33497891351838</v>
+        <v>99.95999999999999</v>
       </c>
       <c r="BK6" t="n">
-        <v>96.86264021536209</v>
+        <v>97.69</v>
       </c>
       <c r="BL6" t="n">
-        <v>99.74050776090651</v>
+        <v>100.52</v>
       </c>
       <c r="BM6" t="n">
-        <v>98.90513544851549</v>
+        <v>101.3</v>
       </c>
       <c r="BN6" t="n">
-        <v>100.2291756081222</v>
+        <v>102.36</v>
       </c>
       <c r="BO6" t="n">
-        <v>100.5489764229486</v>
+        <v>102.94</v>
       </c>
       <c r="BP6" t="n">
-        <v>101.8694601359333</v>
+        <v>104.08</v>
       </c>
       <c r="BQ6" t="n">
         <v>100</v>
       </c>
       <c r="BR6" t="n">
-        <v>98.64812916662981</v>
+        <v>100</v>
       </c>
       <c r="BS6" t="n">
-        <v>97.76091607464529</v>
+        <v>100.47</v>
       </c>
       <c r="BT6" t="n">
-        <v>97.88826331773718</v>
+        <v>99.87</v>
       </c>
       <c r="BU6" t="n">
-        <v>97.12093680399204</v>
+        <v>101.81</v>
       </c>
       <c r="BV6" t="n">
-        <v>96.0540617300815</v>
+        <v>98.31</v>
       </c>
       <c r="BW6" t="n">
-        <v>99.4256844074889</v>
+        <v>101.01</v>
       </c>
       <c r="BX6" t="n">
-        <v>97.48640291783245</v>
+        <v>101.86</v>
       </c>
       <c r="BY6" t="n">
-        <v>98.81257499565136</v>
+        <v>103.45</v>
       </c>
       <c r="BZ6" t="n">
-        <v>99.09418028831743</v>
+        <v>104.65</v>
       </c>
       <c r="CA6" t="n">
-        <v>100.6017914767923</v>
+        <v>105.92</v>
       </c>
       <c r="CB6" t="n">
-        <v>19.26448890751337</v>
+        <v>34.82</v>
       </c>
       <c r="CC6" t="n">
-        <v>103.3585521077478</v>
+        <v>101.47</v>
       </c>
       <c r="CD6" t="n">
         <v>0</v>
@@ -2243,25 +2233,23 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2024-12-24</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Bullish Engulfing</t>
-        </is>
+          <t>2025-08-13</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1</v>
       </c>
       <c r="D7" t="n">
-        <v>0.88</v>
+        <v>0.74</v>
       </c>
       <c r="E7" t="n">
-        <v>99.06990812440016</v>
+        <v>102.4</v>
       </c>
       <c r="F7" t="n">
-        <v>101.658657044476</v>
+        <v>105.37</v>
       </c>
       <c r="G7" t="n">
-        <v>50.59881538942987</v>
+        <v>5.23</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -2270,220 +2258,220 @@
         <v>100</v>
       </c>
       <c r="J7" t="n">
-        <v>102.0151842804438</v>
+        <v>104.03</v>
       </c>
       <c r="K7" t="n">
-        <v>83.46176192683971</v>
+        <v>27.72</v>
       </c>
       <c r="L7" t="n">
         <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>100.4262928488177</v>
+        <v>101.22</v>
       </c>
       <c r="N7" t="n">
-        <v>101.8989279701684</v>
+        <v>105.42</v>
       </c>
       <c r="O7" t="n">
-        <v>3.157776385743426</v>
+        <v>62.52</v>
       </c>
       <c r="P7" t="n">
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>102.0771915881523</v>
+        <v>105.17</v>
       </c>
       <c r="R7" t="n">
-        <v>107.4252065678311</v>
+        <v>106.59</v>
       </c>
       <c r="S7" t="n">
-        <v>113.8738128226098</v>
+        <v>111.76</v>
       </c>
       <c r="T7" t="n">
-        <v>117.1291196038534</v>
+        <v>115.49</v>
       </c>
       <c r="U7" t="n">
-        <v>114.6953889530486</v>
+        <v>118.27</v>
       </c>
       <c r="V7" t="n">
-        <v>0.8913358299464704</v>
+        <v>0.32</v>
       </c>
       <c r="W7" t="n">
-        <v>2.437900505064959</v>
+        <v>0.92</v>
       </c>
       <c r="X7" t="n">
-        <v>5.579978534676422</v>
+        <v>2.1</v>
       </c>
       <c r="Y7" t="n">
-        <v>5.993143621471189</v>
+        <v>3.8</v>
       </c>
       <c r="Z7" t="n">
-        <v>5.889048044184127</v>
+        <v>4.97</v>
       </c>
       <c r="AA7" t="n">
-        <v>99.59695841323737</v>
+        <v>102.98</v>
       </c>
       <c r="AB7" t="n">
-        <v>103.0537919012046</v>
+        <v>106.81</v>
       </c>
       <c r="AC7" t="n">
-        <v>106.9446528897617</v>
+        <v>102.23</v>
       </c>
       <c r="AD7" t="n">
-        <v>116.3772972595798</v>
+        <v>97.38</v>
       </c>
       <c r="AE7" t="n">
-        <v>167.2636685053807</v>
+        <v>75.5</v>
       </c>
       <c r="AF7" t="n">
-        <v>138.5302149980272</v>
+        <v>74.43000000000001</v>
       </c>
       <c r="AG7" t="n">
-        <v>111.7339873275722</v>
+        <v>103.76</v>
       </c>
       <c r="AH7" t="n">
-        <v>105.5272312782544</v>
+        <v>89.11</v>
       </c>
       <c r="AI7" t="n">
-        <v>108.178280479974</v>
+        <v>81.97</v>
       </c>
       <c r="AJ7" t="n">
-        <v>44.76353311619487</v>
+        <v>165.46</v>
       </c>
       <c r="AK7" t="n">
-        <v>65.81461739016069</v>
+        <v>80.72</v>
       </c>
       <c r="AL7" t="n">
-        <v>88.26446536744625</v>
+        <v>83.81</v>
       </c>
       <c r="AM7" t="n">
-        <v>101.0227685928035</v>
+        <v>80.56</v>
       </c>
       <c r="AN7" t="n">
-        <v>95.12676296061335</v>
+        <v>87.44</v>
       </c>
       <c r="AO7" t="n">
-        <v>105.8905570427612</v>
+        <v>105.92</v>
       </c>
       <c r="AP7" t="n">
-        <v>110.0945555265802</v>
+        <v>107.72</v>
       </c>
       <c r="AQ7" t="n">
-        <v>113.7091108639334</v>
+        <v>112.06</v>
       </c>
       <c r="AR7" t="n">
-        <v>112.808862444422</v>
+        <v>107.39</v>
       </c>
       <c r="AS7" t="n">
-        <v>114.3745120753407</v>
+        <v>110.27</v>
       </c>
       <c r="AT7" t="n">
-        <v>114.8910981135847</v>
+        <v>113.26</v>
       </c>
       <c r="AU7" t="n">
-        <v>115.9401617062594</v>
+        <v>113.14</v>
       </c>
       <c r="AV7" t="n">
-        <v>117.015187237115</v>
+        <v>115.21</v>
       </c>
       <c r="AW7" t="n">
-        <v>114.4663581084637</v>
+        <v>114.87</v>
       </c>
       <c r="AX7" t="n">
-        <v>118.0902127679705</v>
+        <v>117.27</v>
       </c>
       <c r="AY7" t="n">
-        <v>115.4076841518286</v>
+        <v>116.25</v>
       </c>
       <c r="AZ7" t="n">
-        <v>112.9677521789188</v>
+        <v>115.36</v>
       </c>
       <c r="BA7" t="n">
-        <v>112.7251555356867</v>
+        <v>115.23</v>
       </c>
       <c r="BB7" t="n">
-        <v>111.9175289798124</v>
+        <v>114.54</v>
       </c>
       <c r="BC7" t="n">
-        <v>107.8197134276038</v>
+        <v>115.34</v>
       </c>
       <c r="BD7" t="n">
-        <v>106.3571497926487</v>
+        <v>113.71</v>
       </c>
       <c r="BE7" t="n">
-        <v>75.60618251767646</v>
+        <v>107.98</v>
       </c>
       <c r="BF7" t="n">
         <v>100</v>
       </c>
       <c r="BG7" t="n">
-        <v>98.19223149680978</v>
+        <v>98.56</v>
       </c>
       <c r="BH7" t="n">
-        <v>100.1749959296692</v>
+        <v>98.12</v>
       </c>
       <c r="BI7" t="n">
-        <v>99.91506872836399</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="BJ7" t="n">
-        <v>100.1629102404349</v>
+        <v>98.33</v>
       </c>
       <c r="BK7" t="n">
-        <v>99.12798720646933</v>
+        <v>96.86</v>
       </c>
       <c r="BL7" t="n">
-        <v>98.85430899687809</v>
+        <v>99.73999999999999</v>
       </c>
       <c r="BM7" t="n">
-        <v>97.16077653018974</v>
+        <v>98.91</v>
       </c>
       <c r="BN7" t="n">
-        <v>96.47353331066559</v>
+        <v>100.23</v>
       </c>
       <c r="BO7" t="n">
-        <v>99.2817947806314</v>
+        <v>100.55</v>
       </c>
       <c r="BP7" t="n">
-        <v>99.54039619395373</v>
+        <v>101.87</v>
       </c>
       <c r="BQ7" t="n">
         <v>100</v>
       </c>
       <c r="BR7" t="n">
-        <v>97.66717976071997</v>
+        <v>98.65000000000001</v>
       </c>
       <c r="BS7" t="n">
-        <v>100.9332642915839</v>
+        <v>97.76000000000001</v>
       </c>
       <c r="BT7" t="n">
-        <v>98.02973854783123</v>
+        <v>97.89</v>
       </c>
       <c r="BU7" t="n">
-        <v>97.39270027759765</v>
+        <v>97.12</v>
       </c>
       <c r="BV7" t="n">
-        <v>95.44556524288518</v>
+        <v>96.05</v>
       </c>
       <c r="BW7" t="n">
-        <v>98.51070710119004</v>
+        <v>99.43000000000001</v>
       </c>
       <c r="BX7" t="n">
-        <v>96.22880798953656</v>
+        <v>97.48999999999999</v>
       </c>
       <c r="BY7" t="n">
-        <v>95.64140953050327</v>
+        <v>98.81</v>
       </c>
       <c r="BZ7" t="n">
-        <v>98.36454742604587</v>
+        <v>99.09</v>
       </c>
       <c r="CA7" t="n">
-        <v>96.92457176926591</v>
+        <v>100.6</v>
       </c>
       <c r="CB7" t="n">
-        <v>19.66198984029427</v>
+        <v>19.26</v>
       </c>
       <c r="CC7" t="n">
-        <v>101.8679184029718</v>
+        <v>103.36</v>
       </c>
       <c r="CD7" t="n">
         <v>0</v>
@@ -2492,7 +2480,7 @@
         <v>0</v>
       </c>
       <c r="CF7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -2503,25 +2491,23 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2024-06-10</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Hammer</t>
-        </is>
+          <t>2024-12-24</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>2</v>
       </c>
       <c r="D8" t="n">
-        <v>0.876</v>
+        <v>0.88</v>
       </c>
       <c r="E8" t="n">
-        <v>102.3552849063574</v>
+        <v>99.06999999999999</v>
       </c>
       <c r="F8" t="n">
-        <v>104.3379934398376</v>
+        <v>101.66</v>
       </c>
       <c r="G8" t="n">
-        <v>65.10051306208973</v>
+        <v>50.6</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -2530,220 +2516,220 @@
         <v>100</v>
       </c>
       <c r="J8" t="n">
-        <v>102.0492360402641</v>
+        <v>102.02</v>
       </c>
       <c r="K8" t="n">
-        <v>26.62359859500324</v>
+        <v>83.45999999999999</v>
       </c>
       <c r="L8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" t="n">
-        <v>99.93346234099464</v>
+        <v>100.43</v>
       </c>
       <c r="N8" t="n">
-        <v>101.4637371281254</v>
+        <v>101.9</v>
       </c>
       <c r="O8" t="n">
-        <v>31.30435936390837</v>
+        <v>3.16</v>
       </c>
       <c r="P8" t="n">
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>104.0851625182829</v>
+        <v>102.08</v>
       </c>
       <c r="R8" t="n">
-        <v>104.9234821997549</v>
+        <v>107.43</v>
       </c>
       <c r="S8" t="n">
-        <v>110.1530234178245</v>
+        <v>113.87</v>
       </c>
       <c r="T8" t="n">
-        <v>104.5508956746562</v>
+        <v>117.13</v>
       </c>
       <c r="U8" t="n">
-        <v>100.7717921746881</v>
+        <v>114.7</v>
       </c>
       <c r="V8" t="n">
-        <v>0.7917514419453866</v>
+        <v>0.89</v>
       </c>
       <c r="W8" t="n">
-        <v>0.8621026222172783</v>
+        <v>2.44</v>
       </c>
       <c r="X8" t="n">
-        <v>1.849593717953805</v>
+        <v>5.58</v>
       </c>
       <c r="Y8" t="n">
-        <v>1.636224523355996</v>
+        <v>5.99</v>
       </c>
       <c r="Z8" t="n">
-        <v>2.064929698256723</v>
+        <v>5.89</v>
       </c>
       <c r="AA8" t="n">
-        <v>100.10645619352</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="AB8" t="n">
-        <v>103.4597450716295</v>
+        <v>103.05</v>
       </c>
       <c r="AC8" t="n">
-        <v>110.1131048833099</v>
+        <v>106.94</v>
       </c>
       <c r="AD8" t="n">
-        <v>107.0392558990244</v>
+        <v>116.38</v>
       </c>
       <c r="AE8" t="n">
-        <v>60.0874213650728</v>
+        <v>167.26</v>
       </c>
       <c r="AF8" t="n">
-        <v>84.64071591009777</v>
+        <v>138.53</v>
       </c>
       <c r="AG8" t="n">
-        <v>91.96373194719277</v>
+        <v>111.73</v>
       </c>
       <c r="AH8" t="n">
-        <v>97.14108508815971</v>
+        <v>105.53</v>
       </c>
       <c r="AI8" t="n">
-        <v>89.29715880563514</v>
+        <v>108.18</v>
       </c>
       <c r="AJ8" t="n">
-        <v>98.20136448211701</v>
+        <v>44.76</v>
       </c>
       <c r="AK8" t="n">
-        <v>143.0269647656458</v>
+        <v>65.81</v>
       </c>
       <c r="AL8" t="n">
-        <v>108.9887474526714</v>
+        <v>88.26000000000001</v>
       </c>
       <c r="AM8" t="n">
-        <v>105.3220709412564</v>
+        <v>101.02</v>
       </c>
       <c r="AN8" t="n">
-        <v>93.73726335686227</v>
+        <v>95.13</v>
       </c>
       <c r="AO8" t="n">
-        <v>104.628074892125</v>
+        <v>105.89</v>
       </c>
       <c r="AP8" t="n">
-        <v>105.6207570694232</v>
+        <v>110.09</v>
       </c>
       <c r="AQ8" t="n">
-        <v>104.2222195375237</v>
+        <v>113.71</v>
       </c>
       <c r="AR8" t="n">
-        <v>105.1124414356419</v>
+        <v>112.81</v>
       </c>
       <c r="AS8" t="n">
-        <v>105.8163660103222</v>
+        <v>114.37</v>
       </c>
       <c r="AT8" t="n">
-        <v>103.4983341727528</v>
+        <v>114.89</v>
       </c>
       <c r="AU8" t="n">
-        <v>106.5202905850025</v>
+        <v>115.94</v>
       </c>
       <c r="AV8" t="n">
-        <v>104.5735158391405</v>
+        <v>117.02</v>
       </c>
       <c r="AW8" t="n">
-        <v>100.0745147669644</v>
+        <v>114.47</v>
       </c>
       <c r="AX8" t="n">
-        <v>102.6267410932785</v>
+        <v>118.09</v>
       </c>
       <c r="AY8" t="n">
-        <v>101.1803023351835</v>
+        <v>115.41</v>
       </c>
       <c r="AZ8" t="n">
-        <v>95.35994396379881</v>
+        <v>112.97</v>
       </c>
       <c r="BA8" t="n">
-        <v>99.73386357708851</v>
+        <v>112.73</v>
       </c>
       <c r="BB8" t="n">
-        <v>95.5755136947883</v>
+        <v>111.92</v>
       </c>
       <c r="BC8" t="n">
-        <v>90.67997142352723</v>
+        <v>107.82</v>
       </c>
       <c r="BD8" t="n">
-        <v>94.91443555527221</v>
+        <v>106.36</v>
       </c>
       <c r="BE8" t="n">
-        <v>71.68882093725105</v>
+        <v>75.61</v>
       </c>
       <c r="BF8" t="n">
         <v>100</v>
       </c>
       <c r="BG8" t="n">
-        <v>99.85393798175373</v>
+        <v>98.19</v>
       </c>
       <c r="BH8" t="n">
-        <v>98.55636695048993</v>
+        <v>100.17</v>
       </c>
       <c r="BI8" t="n">
-        <v>98.95407535437528</v>
+        <v>99.92</v>
       </c>
       <c r="BJ8" t="n">
-        <v>98.9270234590029</v>
+        <v>100.16</v>
       </c>
       <c r="BK8" t="n">
-        <v>97.42370318041027</v>
+        <v>99.13</v>
       </c>
       <c r="BL8" t="n">
-        <v>101.1237102302982</v>
+        <v>98.84999999999999</v>
       </c>
       <c r="BM8" t="n">
-        <v>102.0974509463518</v>
+        <v>97.16</v>
       </c>
       <c r="BN8" t="n">
-        <v>102.024137577378</v>
+        <v>96.47</v>
       </c>
       <c r="BO8" t="n">
-        <v>102.7648858747025</v>
+        <v>99.28</v>
       </c>
       <c r="BP8" t="n">
-        <v>105.0947736284644</v>
+        <v>99.54000000000001</v>
       </c>
       <c r="BQ8" t="n">
         <v>100</v>
       </c>
       <c r="BR8" t="n">
-        <v>99.71962571845782</v>
+        <v>97.67</v>
       </c>
       <c r="BS8" t="n">
-        <v>97.51660594552801</v>
+        <v>100.93</v>
       </c>
       <c r="BT8" t="n">
-        <v>98.6038012002788</v>
+        <v>98.03</v>
       </c>
       <c r="BU8" t="n">
-        <v>97.2296272738173</v>
+        <v>97.39</v>
       </c>
       <c r="BV8" t="n">
-        <v>95.21097749991783</v>
+        <v>95.45</v>
       </c>
       <c r="BW8" t="n">
-        <v>102.0472687979631</v>
+        <v>98.51000000000001</v>
       </c>
       <c r="BX8" t="n">
-        <v>104.3412550860204</v>
+        <v>96.23</v>
       </c>
       <c r="BY8" t="n">
-        <v>103.284255717482</v>
+        <v>95.64</v>
       </c>
       <c r="BZ8" t="n">
-        <v>104.913430780001</v>
+        <v>98.36</v>
       </c>
       <c r="CA8" t="n">
-        <v>108.3918146109794</v>
+        <v>96.92</v>
       </c>
       <c r="CB8" t="n">
-        <v>38.23075618406079</v>
+        <v>19.66</v>
       </c>
       <c r="CC8" t="n">
-        <v>101.3040528378454</v>
+        <v>101.87</v>
       </c>
       <c r="CD8" t="n">
         <v>0</v>
@@ -2752,6 +2738,264 @@
         <v>0</v>
       </c>
       <c r="CF8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SFM</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2024-06-10</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="E9" t="n">
+        <v>102.36</v>
+      </c>
+      <c r="F9" t="n">
+        <v>104.34</v>
+      </c>
+      <c r="G9" t="n">
+        <v>65.09999999999999</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>100</v>
+      </c>
+      <c r="J9" t="n">
+        <v>102.05</v>
+      </c>
+      <c r="K9" t="n">
+        <v>26.62</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>99.93000000000001</v>
+      </c>
+      <c r="N9" t="n">
+        <v>101.46</v>
+      </c>
+      <c r="O9" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>104.09</v>
+      </c>
+      <c r="R9" t="n">
+        <v>104.92</v>
+      </c>
+      <c r="S9" t="n">
+        <v>110.15</v>
+      </c>
+      <c r="T9" t="n">
+        <v>104.55</v>
+      </c>
+      <c r="U9" t="n">
+        <v>100.77</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0.79</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="X9" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>1.64</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>2.06</v>
+      </c>
+      <c r="AA9" t="n">
+        <v>100.11</v>
+      </c>
+      <c r="AB9" t="n">
+        <v>103.46</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>110.11</v>
+      </c>
+      <c r="AD9" t="n">
+        <v>107.04</v>
+      </c>
+      <c r="AE9" t="n">
+        <v>60.09</v>
+      </c>
+      <c r="AF9" t="n">
+        <v>84.64</v>
+      </c>
+      <c r="AG9" t="n">
+        <v>91.95999999999999</v>
+      </c>
+      <c r="AH9" t="n">
+        <v>97.14</v>
+      </c>
+      <c r="AI9" t="n">
+        <v>89.3</v>
+      </c>
+      <c r="AJ9" t="n">
+        <v>98.2</v>
+      </c>
+      <c r="AK9" t="n">
+        <v>143.03</v>
+      </c>
+      <c r="AL9" t="n">
+        <v>108.99</v>
+      </c>
+      <c r="AM9" t="n">
+        <v>105.32</v>
+      </c>
+      <c r="AN9" t="n">
+        <v>93.73999999999999</v>
+      </c>
+      <c r="AO9" t="n">
+        <v>104.63</v>
+      </c>
+      <c r="AP9" t="n">
+        <v>105.62</v>
+      </c>
+      <c r="AQ9" t="n">
+        <v>104.22</v>
+      </c>
+      <c r="AR9" t="n">
+        <v>105.11</v>
+      </c>
+      <c r="AS9" t="n">
+        <v>105.82</v>
+      </c>
+      <c r="AT9" t="n">
+        <v>103.5</v>
+      </c>
+      <c r="AU9" t="n">
+        <v>106.52</v>
+      </c>
+      <c r="AV9" t="n">
+        <v>104.57</v>
+      </c>
+      <c r="AW9" t="n">
+        <v>100.07</v>
+      </c>
+      <c r="AX9" t="n">
+        <v>102.63</v>
+      </c>
+      <c r="AY9" t="n">
+        <v>101.18</v>
+      </c>
+      <c r="AZ9" t="n">
+        <v>95.36</v>
+      </c>
+      <c r="BA9" t="n">
+        <v>99.73</v>
+      </c>
+      <c r="BB9" t="n">
+        <v>95.58</v>
+      </c>
+      <c r="BC9" t="n">
+        <v>90.68000000000001</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>94.91</v>
+      </c>
+      <c r="BE9" t="n">
+        <v>71.69</v>
+      </c>
+      <c r="BF9" t="n">
+        <v>100</v>
+      </c>
+      <c r="BG9" t="n">
+        <v>99.84999999999999</v>
+      </c>
+      <c r="BH9" t="n">
+        <v>98.56</v>
+      </c>
+      <c r="BI9" t="n">
+        <v>98.95</v>
+      </c>
+      <c r="BJ9" t="n">
+        <v>98.93000000000001</v>
+      </c>
+      <c r="BK9" t="n">
+        <v>97.42</v>
+      </c>
+      <c r="BL9" t="n">
+        <v>101.12</v>
+      </c>
+      <c r="BM9" t="n">
+        <v>102.1</v>
+      </c>
+      <c r="BN9" t="n">
+        <v>102.02</v>
+      </c>
+      <c r="BO9" t="n">
+        <v>102.76</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>105.09</v>
+      </c>
+      <c r="BQ9" t="n">
+        <v>100</v>
+      </c>
+      <c r="BR9" t="n">
+        <v>99.72</v>
+      </c>
+      <c r="BS9" t="n">
+        <v>97.52</v>
+      </c>
+      <c r="BT9" t="n">
+        <v>98.59999999999999</v>
+      </c>
+      <c r="BU9" t="n">
+        <v>97.23</v>
+      </c>
+      <c r="BV9" t="n">
+        <v>95.20999999999999</v>
+      </c>
+      <c r="BW9" t="n">
+        <v>102.05</v>
+      </c>
+      <c r="BX9" t="n">
+        <v>104.34</v>
+      </c>
+      <c r="BY9" t="n">
+        <v>103.28</v>
+      </c>
+      <c r="BZ9" t="n">
+        <v>104.91</v>
+      </c>
+      <c r="CA9" t="n">
+        <v>108.39</v>
+      </c>
+      <c r="CB9" t="n">
+        <v>38.23</v>
+      </c>
+      <c r="CC9" t="n">
+        <v>101.3</v>
+      </c>
+      <c r="CD9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CE9" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF9" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>